<commit_message>
Tighten MICE legal applicability outputs
</commit_message>
<xml_diff>
--- a/outputs/may-2026-real-events/details/01-coex-koba-2026/bundle/tables/safety-checklists.xlsx
+++ b/outputs/may-2026-real-events/details/01-coex-koba-2026/bundle/tables/safety-checklists.xlsx
@@ -257,7 +257,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>/Volumes/data/Dev/korea-mice-safety-agent/outputs/may-2026-real-events/details/01-coex-koba-2026</t>
+          <t>outputs/may-2026-real-events/details/01-coex-koba-2026</t>
         </is>
       </c>
     </row>
@@ -1693,7 +1693,7 @@
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:H18"/>
+  <dimension ref="A1:H17"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1998,7 +1998,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>개장 T-75</t>
+          <t>개장 T-60</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -2008,27 +2008,27 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>출입통제·VIP·보안검색</t>
+          <t>등록·CCTV·촬영</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>보안검색 위치, 검색 예외, VIP 동선, 경비원 명부, 경찰·베뉴 보안실 연락 기준 확인</t>
+          <t>개인정보 고지, CCTV 안내판, 촬영 고지, 현장 단말 잠금, 접근권한, 접속기록 담당 확인</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>보안팀장</t>
+          <t>개인정보보호책임자</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>보안 배치표/명부/무전망</t>
+          <t>고지문/안내판 사진/권한 점검표</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>경찰/안전총괄</t>
+          <t>운영총괄/보안책임자</t>
         </is>
       </c>
     </row>
@@ -2040,7 +2040,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>개장 T-60</t>
+          <t>개장 T-45</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -2050,27 +2050,27 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>등록·CCTV·촬영</t>
+          <t>전체 스태프</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>개인정보 고지, CCTV 안내판, 촬영 고지, 현장 단말 잠금, 접근권한, 접속기록 담당 확인</t>
+          <t>안전 브리핑, 구역별 보고선, 무전 채널, 대피/중지/재개 방송문, 미아·분실·민원 처리 기준 공유</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>개인정보보호책임자</t>
+          <t>안전총괄</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>고지문/안내판 사진/권한 점검표</t>
+          <t>브리핑 참석명단/무전 체크</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>운영총괄/보안책임자</t>
+          <t>운영총괄</t>
         </is>
       </c>
     </row>
@@ -2082,7 +2082,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>개장 T-45</t>
+          <t>개장 T-15</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -2092,39 +2092,39 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>전체 스태프</t>
+          <t>운영본부</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>안전 브리핑, 구역별 보고선, 무전 채널, 대피/중지/재개 방송문, 미아·분실·민원 처리 기준 공유</t>
+          <t>개장 승인 hold point: 소방·피난, 의료, 보안, 동선, 전기, 식음료, 작업구역 이상 없음 확인 후 개장</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
+          <t>운영총괄</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>개장 승인 체크/무전 로그</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
           <t>안전총괄</t>
-        </is>
-      </c>
-      <c r="G10" t="inlineStr">
-        <is>
-          <t>브리핑 참석명단/무전 체크</t>
-        </is>
-      </c>
-      <c r="H10" t="inlineStr">
-        <is>
-          <t>운영총괄</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>개장 전</t>
+          <t>운영 중</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>개장 T-15</t>
+          <t>30분 간격</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -2134,39 +2134,39 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>운영본부</t>
+          <t>게이트·혼잡 구역</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>개장 승인 hold point: 소방·피난, 의료, 보안, 동선, 전기, 식음료, 작업구역 이상 없음 확인 후 개장</t>
+          <t>구역별 체류 인원, 대기열 길이, 병목, 우회동선, 스태프 피로도, 위험 신고를 주기 보고</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>운영총괄</t>
+          <t>구역장</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>개장 승인 체크/무전 로그</t>
+          <t>순찰 로그/사진</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>안전총괄</t>
+          <t>안전총괄/보안팀</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>운영 중</t>
+          <t>피크</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>30분 간격</t>
+          <t>피크 T-30~T+30</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -2176,39 +2176,39 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>게이트·혼잡 구역</t>
+          <t>주요 입퇴장 동선</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>구역별 체류 인원, 대기열 길이, 병목, 우회동선, 스태프 피로도, 위험 신고를 주기 보고</t>
+          <t>혼잡 단계 상향 기준, 입장 속도 조절, 우회 안내, 의료·보안 전진 배치, 방송문 준비</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>구역장</t>
+          <t>안전총괄</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>순찰 로그/사진</t>
+          <t>피크 점검 로그/방송 승인</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>안전총괄/보안팀</t>
+          <t>운영총괄/경찰·소방</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>피크</t>
+          <t>폐장</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>피크 T-30~T+30</t>
+          <t>폐장 T-30</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -2218,27 +2218,27 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>주요 입퇴장 동선</t>
+          <t>퇴장 동선</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>혼잡 단계 상향 기준, 입장 속도 조절, 우회 안내, 의료·보안 전진 배치, 방송문 준비</t>
+          <t>퇴장 분산 방송, 역/주차장/셔틀 대기열, 야간 조명, 우회동선, 미아·응급 잔여 이슈 확인</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
+          <t>구역장</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>폐장 전 점검표/방송 로그</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
           <t>안전총괄</t>
-        </is>
-      </c>
-      <c r="G13" t="inlineStr">
-        <is>
-          <t>피크 점검 로그/방송 승인</t>
-        </is>
-      </c>
-      <c r="H13" t="inlineStr">
-        <is>
-          <t>운영총괄/경찰·소방</t>
         </is>
       </c>
     </row>
@@ -2250,7 +2250,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>폐장 T-30</t>
+          <t>폐장 후 T+30</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -2260,39 +2260,39 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>퇴장 동선</t>
+          <t>운영본부</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>퇴장 분산 방송, 역/주차장/셔틀 대기열, 야간 조명, 우회동선, 미아·응급 잔여 이슈 확인</t>
+          <t>사고·응급·민원·분실·미아 기록 취합, 미해결 조치 담당자 지정, 관계기관 종료 공유</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>구역장</t>
+          <t>운영본부 기록담당</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>폐장 전 점검표/방송 로그</t>
+          <t>일일 운영 종료 보고</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>안전총괄</t>
+          <t>운영총괄</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>폐장</t>
+          <t>철거</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>폐장 후 T+30</t>
+          <t>철거 전</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -2302,27 +2302,27 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>운영본부</t>
+          <t>작업구역</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>사고·응급·민원·분실·미아 기록 취합, 미해결 조치 담당자 지정, 관계기관 종료 공유</t>
+          <t>관람객 완전 분리, 전기 차단/투입 승인, 작업허가, PPE, 추락·중량물·화기 작업 통제선 확인</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>운영본부 기록담당</t>
+          <t>작업책임자</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>일일 운영 종료 보고</t>
+          <t>작업허가/교육명단/사진</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>운영총괄</t>
+          <t>안전총괄/베뉴 담당</t>
         </is>
       </c>
     </row>
@@ -2334,7 +2334,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>철거 전</t>
+          <t>철거 중</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -2344,109 +2344,67 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>작업구역</t>
+          <t>하역·반출 동선</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>관람객 완전 분리, 전기 차단/투입 승인, 작업허가, PPE, 추락·중량물·화기 작업 통제선 확인</t>
+          <t>지게차·하역장·차량 동선과 보행동선 분리, 하중분산, 잔재물 낙하·전도 위험 확인</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>작업책임자</t>
+          <t>하역책임자</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>작업허가/교육명단/사진</t>
+          <t>하역 순찰 로그/사진</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>안전총괄/베뉴 담당</t>
+          <t>시설담당/안전총괄</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>철거</t>
+          <t>종료</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>철거 중</t>
+          <t>D+1</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>하역·반출 동선</t>
+          <t>운영본부</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>지게차·하역장·차량 동선과 보행동선 분리, 하중분산, 잔재물 낙하·전도 위험 확인</t>
+          <t>사고보고서, 조치 전후 사진, 제출·승인 증빙, 개인정보 파기/보존, 베뉴 원상복구 확인 정리</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>하역책임자</t>
+          <t>운영본부 기록담당</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>하역 순찰 로그/사진</t>
+          <t>종료 보고서/증빙철</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
-        <is>
-          <t>시설담당/안전총괄</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>종료</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>D+1</t>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>2026-05-13</t>
-        </is>
-      </c>
-      <c r="D18" t="inlineStr">
-        <is>
-          <t>운영본부</t>
-        </is>
-      </c>
-      <c r="E18" t="inlineStr">
-        <is>
-          <t>사고보고서, 조치 전후 사진, 제출·승인 증빙, 개인정보 파기/보존, 베뉴 원상복구 확인 정리</t>
-        </is>
-      </c>
-      <c r="F18" t="inlineStr">
-        <is>
-          <t>운영본부 기록담당</t>
-        </is>
-      </c>
-      <c r="G18" t="inlineStr">
-        <is>
-          <t>종료 보고서/증빙철</t>
-        </is>
-      </c>
-      <c r="H18" t="inlineStr">
         <is>
           <t>운영총괄</t>
         </is>
@@ -2458,7 +2416,7 @@
 
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:G9"/>
+  <dimension ref="A1:G7"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2506,27 +2464,27 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>옥외광고 담당부서/베뉴</t>
+          <t>관할 건축부서/베뉴 시설팀</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>현수막·배너·안내판·전기 광고물 허가/신고</t>
+          <t>가설건축물 축조신고서, 피난안전 확인서, 임시사용승인 확인</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>옥외 임시 안내물, 지주형 표시물, 전광류 또는 전기 사용 광고물을 설치하는 경우</t>
+          <t>대형 텐트, 임시 전시장, 복층/다층 임시구조물, 공사 중 구역 임시 사용</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>표시·설치 전</t>
+          <t>설치 전 신고·승인, 개장 전 피난안전 확인</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>옥외광고물법 시행령 제5·7·12·14조와 관할 조례 확인</t>
+          <t>건축법 시행규칙 별지 제8·8의2·17호서식</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -2543,27 +2501,27 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>관할 건축부서/베뉴 시설팀</t>
+          <t>베뉴 운영/시설/전기/방재 담당</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>가설건축물 축조신고서, 피난안전 확인서, 임시사용승인 확인</t>
+          <t>부스 시공, 전기, 하역, 소방통로, 반입제한, 제출 안전서류</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>대형 텐트, 임시 전시장, 복층/다층 임시구조물, 공사 중 구역 임시 사용</t>
+          <t>전시장·컨벤션센터·공연장 등 베뉴를 사용하는 경우</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>설치 전 신고·승인, 개장 전 피난안전 확인</t>
+          <t>주최자 매뉴얼 기한, 시공 전, 개장 전</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>건축법 시행규칙 별지 제8·8의2·17호서식</t>
+          <t>코엑스 운영규정/안전수칙과 venue-facility sourceSpan 확인</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -2580,27 +2538,27 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>베뉴 운영/시설/전기/방재 담당</t>
+          <t>소방서/베뉴 방재실/안전총괄</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>부스 시공, 전기, 하역, 소방통로, 반입제한, 제출 안전서류</t>
+          <t>소방·피난 점검표, 화기·위험물 반입 승인, 임시소방시설 확인</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>전시장·컨벤션센터·공연장 등 베뉴를 사용하는 경우</t>
+          <t>화기, 위험물, 임시전기, 부스·무대 설치, 피난통로 차단 위험이 있는 경우</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>주최자 매뉴얼 기한, 시공 전, 개장 전</t>
+          <t>설치 전, 개장 전, 피크 전, 철거 전</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>코엑스 운영규정/안전수칙과 venue-facility sourceSpan 확인</t>
+          <t>화재예방법·소방시설법 하위 별표와 베뉴 방재실 승인조건</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -2617,27 +2575,27 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>소방서/베뉴 방재실/안전총괄</t>
+          <t>개인정보 보호책임자/등록 대행사/보안 담당</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>소방·피난 점검표, 화기·위험물 반입 승인, 임시소방시설 확인</t>
+          <t>개인정보 처리방침, 위탁계약, CCTV 안내, 접근권한·접속기록 점검</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>화기, 위험물, 임시전기, 부스·무대 설치, 피난통로 차단 위험이 있는 경우</t>
+          <t>등록, QR/출입증, CCTV, 촬영, 앱 신고, VIP/초청자 명단 처리</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>설치 전, 개장 전, 피크 전, 철거 전</t>
+          <t>수집 전 고지, 행사 전 위탁·보안점검, 종료 후 파기</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>화재예방법·소방시설법 하위 별표와 베뉴 방재실 승인조건</t>
+          <t>개인정보보호법 제15·22·25·26·29·30조와 시행령 안전성 확보 조치</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -2654,27 +2612,27 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>개인정보 보호책임자/등록 대행사/보안 담당</t>
+          <t>의료담당/AED 관리책임자/119·이송병원</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>개인정보 처리방침, 위탁계약, CCTV 안내, 접근권한·접속기록 점검</t>
+          <t>응급의료·AED·구급 이송 계획, AED 점검·교육·관리서류</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>등록, QR/출입증, CCTV, 촬영, 앱 신고, VIP/초청자 명단 처리</t>
+          <t>대규모 인파, 고령자/영유아/장애인, 스탠딩 공연, 야외·폭염·야간 행사</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>수집 전 고지, 행사 전 위탁·보안점검, 종료 후 파기</t>
+          <t>개장 전, 운영 중, 사용/이송 발생 시</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>개인정보보호법 제15·22·25·26·29·30조와 시행령 안전성 확보 조치</t>
+          <t>응급의료법 AED 설치·관리, 시행규칙 구급차 장비·운행기록 기준</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -2691,104 +2649,30 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>경찰/경비업체/베뉴 보안실</t>
+          <t>시공/하역/전기 협력사/안전총괄</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>경비업 허가 범위, 경비지도사, 경비원 명부, 배치·폐지 신고</t>
+          <t>설치·철거 작업자 안전계획서, 작업계획서, 교육명단, PPE·작업중지 기준</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>VIP, 보안검색, 민간경비, 혼잡·교통유도경비를 운영하는 경우</t>
+          <t>부스·무대·트러스·전기·고소·중량물·화기·철거 작업이 있는 경우</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>배치 전, 20일 이상 배치 또는 신고 대상 조건 확인</t>
+          <t>작업 전, 작업 중 변경 시, 철거 전</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>경비업법·시행령·시행규칙 별표/별지 서식</t>
+          <t>산안법, 산안기준규칙 제38·42·321조, KOSHA Guide worker-safety layer</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
-        <is>
-          <t>open</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>7</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>의료담당/AED 관리책임자/119·이송병원</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>응급의료·AED·구급 이송 계획, AED 점검·교육·관리서류</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>대규모 인파, 고령자/영유아/장애인, 스탠딩 공연, 야외·폭염·야간 행사</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>개장 전, 운영 중, 사용/이송 발생 시</t>
-        </is>
-      </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>응급의료법 AED 설치·관리, 시행규칙 구급차 장비·운행기록 기준</t>
-        </is>
-      </c>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t>open</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>8</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>시공/하역/전기 협력사/안전총괄</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>설치·철거 작업자 안전계획서, 작업계획서, 교육명단, PPE·작업중지 기준</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>부스·무대·트러스·전기·고소·중량물·화기·철거 작업이 있는 경우</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>작업 전, 작업 중 변경 시, 철거 전</t>
-        </is>
-      </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>산안법, 산안기준규칙 제38·42·321조, KOSHA Guide worker-safety layer</t>
-        </is>
-      </c>
-      <c r="G9" t="inlineStr">
         <is>
           <t>open</t>
         </is>
@@ -4123,7 +4007,7 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>536</t>
+          <t>365</t>
         </is>
       </c>
     </row>
@@ -4155,7 +4039,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>544</t>
+          <t>373</t>
         </is>
       </c>
     </row>
@@ -4187,7 +4071,7 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>542</t>
+          <t>371</t>
         </is>
       </c>
     </row>
@@ -4219,7 +4103,7 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>246</t>
+          <t>116</t>
         </is>
       </c>
     </row>
@@ -4251,7 +4135,7 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>665</t>
+          <t>494</t>
         </is>
       </c>
     </row>
@@ -4315,7 +4199,7 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>704</t>
+          <t>533</t>
         </is>
       </c>
     </row>
@@ -4347,7 +4231,7 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>708</t>
+          <t>537</t>
         </is>
       </c>
     </row>
@@ -4379,7 +4263,7 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>254</t>
+          <t>124</t>
         </is>
       </c>
     </row>
@@ -4411,7 +4295,7 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>253</t>
+          <t>123</t>
         </is>
       </c>
     </row>
@@ -4443,7 +4327,7 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>778</t>
+          <t>607</t>
         </is>
       </c>
     </row>
@@ -4475,7 +4359,7 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>662</t>
+          <t>491</t>
         </is>
       </c>
     </row>
@@ -4539,7 +4423,7 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>814</t>
+          <t>643</t>
         </is>
       </c>
     </row>
@@ -4571,7 +4455,7 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>841</t>
+          <t>669</t>
         </is>
       </c>
     </row>
@@ -4603,7 +4487,7 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>354</t>
+          <t>224</t>
         </is>
       </c>
     </row>
@@ -4635,7 +4519,7 @@
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>869</t>
+          <t>695</t>
         </is>
       </c>
     </row>
@@ -7260,7 +7144,7 @@
 
 <file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:M9"/>
+  <dimension ref="A1:M7"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7338,17 +7222,17 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>옥외광고 담당부서/베뉴</t>
+          <t>관할 건축부서/베뉴 시설팀</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>현수막·배너·안내판·전기 광고물 허가/신고</t>
+          <t>가설건축물 축조신고서, 피난안전 확인서, 임시사용승인 확인</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>local_government | venue</t>
+          <t>local_government | venue | fire_police_medical</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -7388,7 +7272,7 @@
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>광고물 허가·신고필증/베뉴 설치 승인/설치 사진</t>
+          <t>가설건축물 신고필증/피난안전 확인서/임시사용 승인 확인</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
@@ -7405,32 +7289,32 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>관할 건축부서/베뉴 시설팀</t>
+          <t>베뉴 운영/시설/전기/방재 담당</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>가설건축물 축조신고서, 피난안전 확인서, 임시사용승인 확인</t>
+          <t>부스 시공, 전기, 하역, 소방통로, 반입제한, 제출 안전서류</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>local_government | venue | fire_police_medical</t>
+          <t>venue | fire_police_medical | worker_contractor</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>T-7 설치·작업 전 승인</t>
+          <t>T-1 개장 전 확인</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>2026-05-11 개장 전 현장 확인</t>
+          <t>2026-05-12 운영 중 재점검</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
@@ -7455,7 +7339,7 @@
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>가설건축물 신고필증/피난안전 확인서/임시사용 승인 확인</t>
+          <t>소방·피난 점검표/위험물 반입 승인/개장 전 사진</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
@@ -7472,12 +7356,12 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>베뉴 운영/시설/전기/방재 담당</t>
+          <t>소방서/베뉴 방재실/안전총괄</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>부스 시공, 전기, 하역, 소방통로, 반입제한, 제출 안전서류</t>
+          <t>소방·피난 점검표, 화기·위험물 반입 승인, 임시소방시설 확인</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -7487,17 +7371,17 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>T-1 개장 전 확인</t>
+          <t>T-7 설치·작업 전 승인</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-05</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>2026-05-12 운영 중 재점검</t>
+          <t>2026-05-11 개장 전 현장 확인</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -7539,57 +7423,57 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>소방서/베뉴 방재실/안전총괄</t>
+          <t>개인정보 보호책임자/등록 대행사/보안 담당</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>소방·피난 점검표, 화기·위험물 반입 승인, 임시소방시설 확인</t>
+          <t>개인정보 처리방침, 위탁계약, CCTV 안내, 접근권한·접속기록 점검</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>venue | fire_police_medical | worker_contractor</t>
+          <t>local_government | privacy_security</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>T-7 설치·작업 전 승인</t>
+          <t>T-14 사전점검</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-04-28</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2026-05-11 개장 전 현장 확인</t>
+          <t>2026-05-11 고지·권한 최종 확인</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>시설·방재 담당</t>
+          <t>개인정보보호책임자</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>안전총괄</t>
+          <t>개인정보보호책임자</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>소방서/베뉴 방재실/시설팀</t>
+          <t>등록 대행사/보안 담당</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>운영본부/구역장</t>
+          <t>운영본부</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>소방·피난 점검표/위험물 반입 승인/개장 전 사진</t>
+          <t>처리방침/위탁계약/안내문/CCTV 고지 사진/접속기록 점검표</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
@@ -7606,57 +7490,57 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>개인정보 보호책임자/등록 대행사/보안 담당</t>
+          <t>의료담당/AED 관리책임자/119·이송병원</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>개인정보 처리방침, 위탁계약, CCTV 안내, 접근권한·접속기록 점검</t>
+          <t>응급의료·AED·구급 이송 계획, AED 점검·교육·관리서류</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>local_government | privacy_security</t>
+          <t>fire_police_medical</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>T-14 사전점검</t>
+          <t>T-1 개장 전 확인</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>2026-04-28</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>2026-05-11 고지·권한 최종 확인</t>
+          <t>2026-05-12 운영 중 재점검</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>개인정보보호책임자</t>
+          <t>의료담당</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>개인정보보호책임자</t>
+          <t>안전총괄</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>등록 대행사/보안 담당</t>
+          <t>119/이송병원/AED 관리책임자</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>운영본부</t>
+          <t>운영본부/구역장</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>처리방침/위탁계약/안내문/CCTV 고지 사진/접속기록 점검표</t>
+          <t>AED 점검표/응급인력 배치표/119·이송병원 협의 기록</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
@@ -7673,22 +7557,22 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>경찰/경비업체/베뉴 보안실</t>
+          <t>시공/하역/전기 협력사/안전총괄</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>경비업 허가 범위, 경비지도사, 경비원 명부, 배치·폐지 신고</t>
+          <t>설치·철거 작업자 안전계획서, 작업계획서, 교육명단, PPE·작업중지 기준</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>local_government | venue | fire_police_medical | privacy_security</t>
+          <t>venue | worker_contractor</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>T-7 담당기관 확인</t>
+          <t>T-7 설치·작업 전 승인</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -7698,12 +7582,12 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>2026-05-11 최종 확인</t>
+          <t>2026-05-11 개장 전 현장 확인</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>교통·대외협력 담당</t>
+          <t>작업책임자</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
@@ -7713,154 +7597,20 @@
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>도로관리청/경찰/지자체</t>
+          <t>시공/하역/전기 협력사</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>운영본부/안내팀</t>
+          <t>운영본부/구역장</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>제출본 PDF/접수증/승인메일/담당자 확인 메모</t>
+          <t>작업계획서/교육명단/PPE 지급/작업허가·작업중지 기준</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
-        <is>
-          <t>open</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>7</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>의료담당/AED 관리책임자/119·이송병원</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>응급의료·AED·구급 이송 계획, AED 점검·교육·관리서류</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>fire_police_medical</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>T-1 개장 전 확인</t>
-        </is>
-      </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>2026-05-11</t>
-        </is>
-      </c>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t>2026-05-12 운영 중 재점검</t>
-        </is>
-      </c>
-      <c r="H8" t="inlineStr">
-        <is>
-          <t>의료담당</t>
-        </is>
-      </c>
-      <c r="I8" t="inlineStr">
-        <is>
-          <t>안전총괄</t>
-        </is>
-      </c>
-      <c r="J8" t="inlineStr">
-        <is>
-          <t>119/이송병원/AED 관리책임자</t>
-        </is>
-      </c>
-      <c r="K8" t="inlineStr">
-        <is>
-          <t>운영본부/구역장</t>
-        </is>
-      </c>
-      <c r="L8" t="inlineStr">
-        <is>
-          <t>AED 점검표/응급인력 배치표/119·이송병원 협의 기록</t>
-        </is>
-      </c>
-      <c r="M8" t="inlineStr">
-        <is>
-          <t>open</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>8</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>시공/하역/전기 협력사/안전총괄</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>설치·철거 작업자 안전계획서, 작업계획서, 교육명단, PPE·작업중지 기준</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>venue | worker_contractor</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>T-7 설치·작업 전 승인</t>
-        </is>
-      </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>2026-05-05</t>
-        </is>
-      </c>
-      <c r="G9" t="inlineStr">
-        <is>
-          <t>2026-05-11 개장 전 현장 확인</t>
-        </is>
-      </c>
-      <c r="H9" t="inlineStr">
-        <is>
-          <t>작업책임자</t>
-        </is>
-      </c>
-      <c r="I9" t="inlineStr">
-        <is>
-          <t>안전총괄</t>
-        </is>
-      </c>
-      <c r="J9" t="inlineStr">
-        <is>
-          <t>시공/하역/전기 협력사</t>
-        </is>
-      </c>
-      <c r="K9" t="inlineStr">
-        <is>
-          <t>운영본부/구역장</t>
-        </is>
-      </c>
-      <c r="L9" t="inlineStr">
-        <is>
-          <t>작업계획서/교육명단/PPE 지급/작업허가·작업중지 기준</t>
-        </is>
-      </c>
-      <c r="M9" t="inlineStr">
         <is>
           <t>open</t>
         </is>

</xml_diff>